<commit_message>
chore: refresh final 99 live evidence
</commit_message>
<xml_diff>
--- a/evaluation/final-99-gate-current-2026-07-21/orchestration-download/files/세이프건설-risk-assessment.xlsx
+++ b/evaluation/final-99-gate-current-2026-07-21/orchestration-download/files/세이프건설-risk-assessment.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="146">
   <si>
     <t>위험성평가표  ·  SafeClaw 안전 양식</t>
   </si>
@@ -64,7 +64,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>위험성평가표(초안)</t>
+    <t>위험성평가표(구조화 편집본)</t>
   </si>
   <si>
     <t>□</t>
@@ -73,238 +73,202 @@
     <t>______</t>
   </si>
   <si>
-    <t>공식자료 기반</t>
-  </si>
-  <si>
-    <t>KOSHA 위험성평가 절차 및 4M 기법 참고</t>
-  </si>
-  <si>
-    <t>업체명</t>
-  </si>
-  <si>
-    <t>업종</t>
-  </si>
-  <si>
-    <t>건설업</t>
-  </si>
-  <si>
-    <t>작업명</t>
+    <t>1. 외벽 도장 작업</t>
+  </si>
+  <si>
+    <t>관리번호</t>
+  </si>
+  <si>
+    <t>RA-construction-painting-1</t>
+  </si>
+  <si>
+    <t>작업장소</t>
+  </si>
+  <si>
+    <t>공정</t>
+  </si>
+  <si>
+    <t>이동식 비계 사용 외벽 도장, 자재 상하차, 하부 통제</t>
+  </si>
+  <si>
+    <t>세부작업</t>
   </si>
   <si>
     <t>외벽 도장 작업</t>
   </si>
   <si>
-    <t>공정/세부작업</t>
-  </si>
-  <si>
-    <t>이동식 비계 사용 외벽 도장, 자재 상하차, 하부 통제</t>
-  </si>
-  <si>
-    <t>작업장소</t>
-  </si>
-  <si>
-    <t>작업인원</t>
-  </si>
-  <si>
-    <t>5명</t>
-  </si>
-  <si>
-    <t>기상 및 작업조건</t>
-  </si>
-  <si>
-    <t>오후 강풍 예보, 작업중지 기준 공유 필요</t>
-  </si>
-  <si>
-    <t>1. 사전준비</t>
-  </si>
-  <si>
-    <t>- 평가대상 작업</t>
-  </si>
-  <si>
-    <t>- 참여자</t>
-  </si>
-  <si>
-    <t>현장소장, 관리감독자, 작업반장, 해당 작업자</t>
-  </si>
-  <si>
-    <t>- 확인자료</t>
-  </si>
-  <si>
-    <t>작업계획, 기상조건, 장비·보호구 상태, 최근 TBM 기록</t>
-  </si>
-  <si>
-    <t>2. 유해·위험요인 파악</t>
-  </si>
-  <si>
-    <t>1. 세부작업</t>
+    <t>장비/도구</t>
+  </si>
+  <si>
+    <t>이동식 비계, 안전난간, 추락방지 보호구</t>
+  </si>
+  <si>
+    <t>유해·위험요인</t>
   </si>
   <si>
     <t>이동식 비계 승·하강 및 작업발판 이동 중 추락</t>
   </si>
   <si>
+    <t>4M</t>
+  </si>
+  <si>
+    <t>Machine</t>
+  </si>
+  <si>
+    <t>재해형태</t>
+  </si>
+  <si>
+    <t>fall</t>
+  </si>
+  <si>
+    <t>현재 안전조치</t>
+  </si>
+  <si>
+    <t>작업 전 비계 고정핀, 바퀴 잠금, 작업발판 상태 점검</t>
+  </si>
+  <si>
+    <t>가능성</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>중대성</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>위험등급</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>추가 감소대책</t>
+  </si>
+  <si>
+    <t>조치담당자</t>
+  </si>
+  <si>
+    <t>관리감독자</t>
+  </si>
+  <si>
+    <t>조치기한</t>
+  </si>
+  <si>
+    <t>현장 확인</t>
+  </si>
+  <si>
+    <t>확인방법</t>
+  </si>
+  <si>
+    <t>작업 전 TBM 및 현장 사진 확인</t>
+  </si>
+  <si>
+    <t>planned</t>
+  </si>
+  <si>
+    <t>확인일</t>
+  </si>
+  <si>
+    <t>확인자</t>
+  </si>
+  <si>
+    <t>작업반장</t>
+  </si>
+  <si>
+    <t>가능성 판단근거</t>
+  </si>
+  <si>
+    <t>작업 전 노출 빈도와 현장 통제 상태를 함께 반영</t>
+  </si>
+  <si>
+    <t>중대성 판단근거</t>
+  </si>
+  <si>
+    <t>추락·충돌·화재 등 중대재해 가능성을 보수적으로 반영</t>
+  </si>
+  <si>
+    <t>근거</t>
+  </si>
+  <si>
+    <t>riskAssessmentDraft | tbmBriefing</t>
+  </si>
+  <si>
+    <t>2. 강풍 시 비계 전도와 공구·자재 낙하</t>
+  </si>
+  <si>
+    <t>RA-construction-painting-2</t>
+  </si>
+  <si>
+    <t>강풍 시 비계 전도와 공구·자재 낙하</t>
+  </si>
+  <si>
+    <t>풍속 상승 또는 돌풍 체감 시 즉시 작업중지 후 지상 대기</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>작업 전 체크리스트 확인</t>
+  </si>
+  <si>
+    <t>needsReview</t>
+  </si>
+  <si>
+    <t>3. 지게차 동선 인접 구간에서 작업자 충돌</t>
+  </si>
+  <si>
+    <t>RA-construction-painting-3</t>
+  </si>
+  <si>
+    <t>지게차 동선 인접 구간에서 작업자 충돌</t>
+  </si>
+  <si>
+    <t>지게차, 랙, 팔레트, 신호장비</t>
+  </si>
+  <si>
+    <t>struckBy</t>
+  </si>
+  <si>
+    <t>작업반장 주도로 보호구 착용과 작업구간 출입통제를 확인</t>
+  </si>
+  <si>
+    <t>공식 서식 기준 보강</t>
+  </si>
+  <si>
+    <t>KOSHA 위험성평가 흐름에 맞춰 사전준비, 유해·위험요인 파악, 위험성 결정, 감소대책, 공유·교육, 조치 확인 순서로 기록합니다.</t>
+  </si>
+  <si>
+    <t>4M 관점(작업자, 장비·도구, 작업환경, 관리체계)을 누락 점검 기준으로 사용합니다.</t>
+  </si>
+  <si>
+    <t>- 반영 근거</t>
+  </si>
+  <si>
+    <t>KOSHA 위험성평가 사업안내 / KOSHA 위험성평가 교육자료 / 지게차의 안전작업에 관한 기술지원규정</t>
+  </si>
+  <si>
+    <t>옥외작업 폭염·자외선 위험 반영</t>
+  </si>
+  <si>
+    <t>- 폭염·고온 신호</t>
+  </si>
+  <si>
+    <t>영향예보 보건(일반인) 주의 (부산동부)</t>
+  </si>
+  <si>
+    <t>- 자외선 신호</t>
+  </si>
+  <si>
+    <t>자외선지수 1 (낮음) / 실시간 홍반자외선 연결 보류</t>
+  </si>
+  <si>
     <t>- 유해·위험요인</t>
-  </si>
-  <si>
-    <t>- 4M 체크</t>
-  </si>
-  <si>
-    <t>Man:■ Machine:■ Media:□ Management:□ / 중점 확인: Man, Machine</t>
-  </si>
-  <si>
-    <t>2. 세부작업</t>
-  </si>
-  <si>
-    <t>강풍 시 비계 전도와 공구·자재 낙하</t>
-  </si>
-  <si>
-    <t>Man:■ Machine:■ Media:■ Management:□ / 중점 확인: Man, Machine, Media</t>
-  </si>
-  <si>
-    <t>3. 세부작업</t>
-  </si>
-  <si>
-    <t>지게차 동선 인접 구간에서 작업자 충돌</t>
-  </si>
-  <si>
-    <t>Man:■ Machine:■ Media:■ Management:■ / 중점 확인: Man, Machine, Media, Management</t>
-  </si>
-  <si>
-    <t>3. 위험성 결정</t>
-  </si>
-  <si>
-    <t>- 현재 위험성</t>
-  </si>
-  <si>
-    <t>상</t>
-  </si>
-  <si>
-    <t>- 판단근거</t>
-  </si>
-  <si>
-    <t>사고 발생 가능성과 중대성을 함께 고려</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>작업 전 통제 여부와 노출 빈도 확인</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>중</t>
-  </si>
-  <si>
-    <t>관리감독 및 작업자 숙지 여부 확인</t>
-  </si>
-  <si>
-    <t>4. 감소대책 수립 및 실행</t>
-  </si>
-  <si>
-    <t>작업 전 비계 고정핀, 바퀴 잠금, 작업발판 상태 점검</t>
-  </si>
-  <si>
-    <t>- 실행시점</t>
-  </si>
-  <si>
-    <t>작업 시작 전</t>
-  </si>
-  <si>
-    <t>- 담당</t>
-  </si>
-  <si>
-    <t>관리감독자 / 작업반장</t>
-  </si>
-  <si>
-    <t>- 잔여 위험성</t>
-  </si>
-  <si>
-    <t>풍속 상승 또는 돌풍 체감 시 즉시 작업중지 후 지상 대기</t>
-  </si>
-  <si>
-    <t>작업 시작 전 및 작업 중 수시</t>
-  </si>
-  <si>
-    <t>작업반장 / 신호수</t>
-  </si>
-  <si>
-    <t>작업반장 주도로 보호구 착용과 작업구간 출입통제를 확인</t>
-  </si>
-  <si>
-    <t>TBM 직후</t>
-  </si>
-  <si>
-    <t>전 작업자</t>
-  </si>
-  <si>
-    <t>하</t>
-  </si>
-  <si>
-    <t>5. 공유·교육</t>
-  </si>
-  <si>
-    <t>위험성평가 결과는 TBM에서 구두 설명하고, 작업자 이해 여부를 확인합니다.</t>
-  </si>
-  <si>
-    <t>신규 투입자와 외국인 근로자는 쉬운 문장 또는 다국어 보조 설명을 추가합니다.</t>
-  </si>
-  <si>
-    <t>6. 조치 확인</t>
-  </si>
-  <si>
-    <t>위험성평가 실시자</t>
-  </si>
-  <si>
-    <t>현장소장 / 관리감독자</t>
-  </si>
-  <si>
-    <t>근로자 참여 확인</t>
-  </si>
-  <si>
-    <t>작업 전 TBM에서 공유 및 복창 확인</t>
-  </si>
-  <si>
-    <t>조치 완료 예정일</t>
-  </si>
-  <si>
-    <t>작업 시작 전 즉시</t>
-  </si>
-  <si>
-    <t>미조치 항목 처리</t>
-  </si>
-  <si>
-    <t>작업 보류 또는 책임자 승인 후 재평가</t>
-  </si>
-  <si>
-    <t>공식 서식 기준 보강</t>
-  </si>
-  <si>
-    <t>KOSHA 위험성평가 흐름에 맞춰 사전준비, 유해·위험요인 파악, 위험성 결정, 감소대책, 공유·교육, 조치 확인 순서로 기록합니다.</t>
-  </si>
-  <si>
-    <t>4M 관점(작업자, 장비·도구, 작업환경, 관리체계)을 누락 점검 기준으로 사용합니다.</t>
-  </si>
-  <si>
-    <t>- 반영 근거</t>
-  </si>
-  <si>
-    <t>KOSHA 위험성평가 사업안내 / KOSHA 위험성평가 교육자료 / 지게차의 안전작업에 관한 기술지원규정</t>
-  </si>
-  <si>
-    <t>옥외작업 폭염·자외선 위험 반영</t>
-  </si>
-  <si>
-    <t>- 폭염·고온 신호</t>
-  </si>
-  <si>
-    <t>여름철 체감온도 연결 보류</t>
-  </si>
-  <si>
-    <t>- 자외선 신호</t>
-  </si>
-  <si>
-    <t>자외선지수 1 (낮음) / 실시간 홍반자외선 연결 보류</t>
   </si>
   <si>
     <t>고온 노출, 직사광선, 탈수, 열탈진·열사병, 자외선 노출, 신규·고령·민감군 작업자 상태 악화</t>
@@ -915,7 +879,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1012,13 +976,13 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>18</v>
@@ -1032,13 +996,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>18</v>
@@ -1052,13 +1016,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>18</v>
@@ -1072,13 +1036,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>18</v>
@@ -1092,13 +1056,13 @@
         <v>6</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>18</v>
@@ -1112,13 +1076,13 @@
         <v>7</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>18</v>
@@ -1132,13 +1096,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>18</v>
@@ -1152,13 +1116,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>18</v>
@@ -1172,13 +1136,13 @@
         <v>10</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>18</v>
@@ -1192,13 +1156,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>18</v>
@@ -1212,13 +1176,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>18</v>
@@ -1232,13 +1196,13 @@
         <v>13</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>18</v>
@@ -1252,13 +1216,13 @@
         <v>14</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>18</v>
@@ -1272,13 +1236,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>18</v>
@@ -1292,13 +1256,13 @@
         <v>16</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>18</v>
@@ -1312,13 +1276,13 @@
         <v>17</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>18</v>
@@ -1332,13 +1296,13 @@
         <v>18</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>18</v>
@@ -1352,13 +1316,13 @@
         <v>19</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>18</v>
@@ -1372,13 +1336,13 @@
         <v>20</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>18</v>
@@ -1392,13 +1356,13 @@
         <v>21</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>18</v>
@@ -1412,13 +1376,13 @@
         <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>18</v>
@@ -1432,13 +1396,13 @@
         <v>23</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>18</v>
@@ -1452,13 +1416,13 @@
         <v>24</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>18</v>
@@ -1472,13 +1436,13 @@
         <v>25</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>18</v>
@@ -1492,13 +1456,13 @@
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>18</v>
@@ -1512,13 +1476,13 @@
         <v>27</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>18</v>
@@ -1532,13 +1496,13 @@
         <v>28</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>18</v>
@@ -1552,13 +1516,13 @@
         <v>29</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>18</v>
@@ -1572,13 +1536,13 @@
         <v>30</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>18</v>
@@ -1592,13 +1556,13 @@
         <v>31</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>18</v>
@@ -1612,13 +1576,13 @@
         <v>32</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C37" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>18</v>
@@ -1632,13 +1596,13 @@
         <v>33</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>18</v>
@@ -1652,13 +1616,13 @@
         <v>34</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>18</v>
@@ -1672,13 +1636,13 @@
         <v>35</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>18</v>
@@ -1692,13 +1656,13 @@
         <v>36</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>18</v>
@@ -1712,13 +1676,13 @@
         <v>37</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>18</v>
@@ -1732,13 +1696,13 @@
         <v>38</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>18</v>
@@ -1752,13 +1716,13 @@
         <v>39</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>18</v>
@@ -1772,13 +1736,13 @@
         <v>40</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>64</v>
+        <v>13</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>18</v>
@@ -1792,13 +1756,13 @@
         <v>41</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>18</v>
@@ -1812,13 +1776,13 @@
         <v>42</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="E47" s="4" t="s">
         <v>18</v>
@@ -1832,13 +1796,13 @@
         <v>43</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>18</v>
@@ -1852,13 +1816,13 @@
         <v>44</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>57</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>18</v>
@@ -1872,13 +1836,13 @@
         <v>45</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>18</v>
@@ -1892,13 +1856,13 @@
         <v>46</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>18</v>
@@ -1912,13 +1876,13 @@
         <v>47</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>18</v>
@@ -1932,13 +1896,13 @@
         <v>48</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>87</v>
+        <v>25</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>18</v>
@@ -1952,13 +1916,13 @@
         <v>49</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>18</v>
@@ -1972,13 +1936,13 @@
         <v>50</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>18</v>
@@ -1992,13 +1956,13 @@
         <v>51</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E56" s="4" t="s">
         <v>18</v>
@@ -2012,13 +1976,13 @@
         <v>52</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="E57" s="4" t="s">
         <v>18</v>
@@ -2032,13 +1996,13 @@
         <v>53</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>18</v>
@@ -2052,13 +2016,13 @@
         <v>54</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>18</v>
@@ -2072,13 +2036,13 @@
         <v>55</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>18</v>
@@ -2092,13 +2056,13 @@
         <v>56</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>101</v>
+        <v>40</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>18</v>
@@ -2112,13 +2076,13 @@
         <v>57</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>103</v>
+        <v>42</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>18</v>
@@ -2132,13 +2096,13 @@
         <v>58</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>18</v>
@@ -2152,13 +2116,13 @@
         <v>59</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>18</v>
@@ -2172,13 +2136,13 @@
         <v>60</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>111</v>
+        <v>47</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>112</v>
+        <v>48</v>
       </c>
       <c r="E65" s="4" t="s">
         <v>18</v>
@@ -2192,13 +2156,13 @@
         <v>61</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>113</v>
+        <v>49</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>114</v>
+        <v>67</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>18</v>
@@ -2212,13 +2176,13 @@
         <v>62</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>18</v>
@@ -2232,13 +2196,13 @@
         <v>63</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>18</v>
@@ -2252,13 +2216,13 @@
         <v>64</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>118</v>
+        <v>69</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>119</v>
+        <v>53</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>120</v>
+        <v>54</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>18</v>
@@ -2272,13 +2236,13 @@
         <v>65</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>118</v>
+        <v>69</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>18</v>
@@ -2292,13 +2256,13 @@
         <v>66</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>123</v>
+        <v>69</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>124</v>
+        <v>57</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>125</v>
+        <v>58</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>18</v>
@@ -2312,13 +2276,13 @@
         <v>67</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>123</v>
+        <v>69</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>124</v>
+        <v>59</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>126</v>
+        <v>60</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>18</v>
@@ -2332,13 +2296,13 @@
         <v>68</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>18</v>
@@ -2352,13 +2316,13 @@
         <v>69</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>130</v>
+        <v>77</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>18</v>
@@ -2372,13 +2336,13 @@
         <v>70</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>127</v>
+        <v>75</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>128</v>
+        <v>78</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>18</v>
@@ -2392,13 +2356,13 @@
         <v>71</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>132</v>
+        <v>80</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>134</v>
+        <v>82</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>18</v>
@@ -2412,13 +2376,13 @@
         <v>72</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>132</v>
+        <v>80</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>135</v>
+        <v>84</v>
       </c>
       <c r="E77" s="4" t="s">
         <v>18</v>
@@ -2432,13 +2396,13 @@
         <v>73</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>137</v>
+        <v>85</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>138</v>
+        <v>86</v>
       </c>
       <c r="E78" s="4" t="s">
         <v>18</v>
@@ -2452,13 +2416,13 @@
         <v>74</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>139</v>
+        <v>87</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>140</v>
+        <v>88</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>18</v>
@@ -2472,13 +2436,13 @@
         <v>75</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>139</v>
+        <v>89</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>141</v>
+        <v>90</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>18</v>
@@ -2492,13 +2456,13 @@
         <v>76</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>142</v>
+        <v>91</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>143</v>
+        <v>92</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>18</v>
@@ -2512,13 +2476,13 @@
         <v>77</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>136</v>
+        <v>93</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>142</v>
+        <v>94</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="E82" s="4" t="s">
         <v>18</v>
@@ -2532,13 +2496,13 @@
         <v>78</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>136</v>
+        <v>93</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>142</v>
+        <v>96</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="E83" s="4" t="s">
         <v>18</v>
@@ -2552,13 +2516,13 @@
         <v>79</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>142</v>
+        <v>99</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>146</v>
+        <v>100</v>
       </c>
       <c r="E84" s="4" t="s">
         <v>18</v>
@@ -2572,13 +2536,13 @@
         <v>80</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>142</v>
+        <v>101</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>147</v>
+        <v>102</v>
       </c>
       <c r="E85" s="4" t="s">
         <v>18</v>
@@ -2592,13 +2556,13 @@
         <v>81</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>18</v>
@@ -2612,13 +2576,13 @@
         <v>82</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>136</v>
+        <v>98</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>142</v>
+        <v>16</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>149</v>
+        <v>105</v>
       </c>
       <c r="E87" s="4" t="s">
         <v>18</v>
@@ -2632,13 +2596,13 @@
         <v>83</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>150</v>
+        <v>107</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>151</v>
+        <v>108</v>
       </c>
       <c r="E88" s="4" t="s">
         <v>18</v>
@@ -2652,13 +2616,13 @@
         <v>84</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>150</v>
+        <v>109</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="E89" s="4" t="s">
         <v>18</v>
@@ -2672,13 +2636,13 @@
         <v>85</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>153</v>
+        <v>113</v>
       </c>
       <c r="E90" s="4" t="s">
         <v>18</v>
@@ -2692,13 +2656,13 @@
         <v>86</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="E91" s="4" t="s">
         <v>18</v>
@@ -2712,13 +2676,13 @@
         <v>87</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>155</v>
+        <v>117</v>
       </c>
       <c r="E92" s="4" t="s">
         <v>18</v>
@@ -2732,13 +2696,13 @@
         <v>88</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>156</v>
+        <v>118</v>
       </c>
       <c r="E93" s="4" t="s">
         <v>18</v>
@@ -2752,18 +2716,398 @@
         <v>89</v>
       </c>
       <c r="B94" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>90</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F95" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>91</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>92</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>93</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D98" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>94</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F99" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>95</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>96</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" s="4">
+        <v>97</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D102" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" s="4">
+        <v>98</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E103" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F103" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" s="4">
+        <v>99</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" s="4">
+        <v>100</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D105" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C94" s="6" t="s">
+      <c r="E105" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A106" s="4">
+        <v>101</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D106" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F106" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A107" s="4">
+        <v>102</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F107" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A108" s="4">
+        <v>103</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D108" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E108" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F108" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A109" s="4">
+        <v>104</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D109" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F109" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A110" s="4">
+        <v>105</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D110" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F110" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A111" s="4">
+        <v>106</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D111" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E111" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F111" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A112" s="4">
+        <v>107</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D112" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F112" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A113" s="4">
+        <v>108</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C113" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D94" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="E94" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F94" s="5" t="s">
+      <c r="D113" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F113" s="5" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>